<commit_message>
ios: didascalie degli screenshot nel foglio dello store, prompt ChatGPT aggiornato
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ios/localizzazione/NEAT_store_da_tradurre.xlsx
+++ b/ios/localizzazione/NEAT_store_da_tradurre.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -111,6 +111,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -531,6 +532,13 @@
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Esempio: store.subtitle · Italiano «Il tuo obiettivo. Raggiungilo.» · Inglese «Set a goal. Reach it.»</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Didascalie degli screenshot (righe shot*): titoli brevissimi in MAIUSCOLO su 2 righe, sottotitoli corti. Contano la lunghezza e il ritmo, non la traduzione letterale. Per JA/KO/ZH ignora il MAIUSCOLO.</t>
         </is>
       </c>
     </row>
@@ -545,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -845,6 +853,576 @@
       <c r="O6" s="6" t="n"/>
       <c r="P6" s="6" t="n"/>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>shot1.title</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 1 · titolo</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>≤ 32</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Didascalia grande in alto, MAIUSCOLO, carattere Anton stretto, su 2 righe. Prima immagine: la domanda principale. Sotto c'è la Home con i passi di oggi.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>QUANTI PASSI HAI FATTO OGGI?</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="n"/>
+      <c r="M7" s="6" t="n"/>
+      <c r="N7" s="6" t="n"/>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>shot1.sub</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 1 · sottotitolo</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>≤ 34</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Riga piccola in un'etichetta nera sotto il titolo.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Datti un obiettivo e controllalo</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n"/>
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="6" t="n"/>
+      <c r="M8" s="6" t="n"/>
+      <c r="N8" s="6" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>shot2.title</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 2 · titolo</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>≤ 32</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>MAIUSCOLO, 2 righe. Sotto: i minuti di camminata che mancano.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>QUANTI TE NE MANCANO?</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="n"/>
+      <c r="M9" s="6" t="n"/>
+      <c r="N9" s="6" t="n"/>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>shot2.sub</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 2 · sottotitolo</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>≤ 38</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Etichetta rossa.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>In minuti di camminata e chilometri</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="6" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>shot3.title</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 3 · titolo</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>≤ 32</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>MAIUSCOLO, 2 righe. Sotto: lo stesso giorno a 4 e a 16 km/h, i minuti cambiano.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>QUANTO DEVI ANCORA CAMMINARE?</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
+      <c r="M11" s="6" t="n"/>
+      <c r="N11" s="6" t="n"/>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>shot3.sub</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 3 · sottotitolo</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>≤ 28</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Etichetta nera.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Alla velocità che scegli</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="6" t="n"/>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>shot4.title</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 4 · titolo</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>≤ 32</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>MAIUSCOLO, 2 righe. Sotto: lo Storico con la serie (glossario).</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>OGNI GIORNO ALLUNGA LA SERIE</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="6" t="n"/>
+      <c r="O13" s="6" t="n"/>
+      <c r="P13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>shot4.sub</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 4 · sottotitolo</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>≤ 40</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Etichetta nera. «Jolly» secondo il glossario.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Ogni 15 giorni di fila arriva un Jolly</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="6" t="n"/>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>shot5.title</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 5 · titolo</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>≤ 32</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>MAIUSCOLO, 2 righe. Sotto: i widget.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>SEMPRE SOTTO GLI OCCHI</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
+      <c r="M15" s="6" t="n"/>
+      <c r="N15" s="6" t="n"/>
+      <c r="O15" s="6" t="n"/>
+      <c r="P15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>shot5.sub</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 5 · sottotitolo</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>≤ 34</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Etichetta rossa. «Home» = schermata Home di iOS, «blocco schermo» = Lock Screen (nomi ufficiali Apple nella lingua).</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Widget per Home e blocco schermo</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n"/>
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="6" t="n"/>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>shot6.title</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 6 · titolo</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>≤ 36</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>MAIUSCOLO, 2 righe. La promessa sulla privacy (stessa del testo promozionale).</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>I TUOI DATI RESTANO SUL TUO IPHONE</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="M17" s="6" t="n"/>
+      <c r="N17" s="6" t="n"/>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>shot6.sub</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 6 · sottotitolo</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>≤ 34</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Etichetta nera.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Niente account, niente pubblicità</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
+      <c r="M18" s="6" t="n"/>
+      <c r="N18" s="6" t="n"/>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>shot6.tag1</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 6 · etichetta 1</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>≤ 20</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Etichetta nera MAIUSCOLA sopra l'immagine.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>NIENTE ACCOUNT</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+      <c r="M19" s="6" t="n"/>
+      <c r="N19" s="6" t="n"/>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>shot6.tag2</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 6 · etichetta 2</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>≤ 20</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Etichetta nera MAIUSCOLA.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>NIENTE PUBBLICITÀ</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+      <c r="M20" s="6" t="n"/>
+      <c r="N20" s="6" t="n"/>
+      <c r="O20" s="6" t="n"/>
+      <c r="P20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>shot6.tag3</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot 6 · etichetta 3</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>≤ 20</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Etichetta nera MAIUSCOLA.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>NIENTE TRACCIAMENTO</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
+      <c r="M21" s="6" t="n"/>
+      <c r="N21" s="6" t="n"/>
+      <c r="O21" s="6" t="n"/>
+      <c r="P21" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ios: didascalia 6 senza ripetizioni, a capo dei titoli segnati con /
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ios/localizzazione/NEAT_store_da_tradurre.xlsx
+++ b/ios/localizzazione/NEAT_store_da_tradurre.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -539,6 +539,13 @@
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Didascalie degli screenshot (righe shot*): titoli brevissimi in MAIUSCOLO su 2 righe, sottotitoli corti. Contano la lunghezza e il ritmo, non la traduzione letterale. Per JA/KO/ZH ignora il MAIUSCOLO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Titoli degli screenshot: segna l'a capo con « / » (una sola barra, al massimo 2 righe).</t>
         </is>
       </c>
     </row>
@@ -871,7 +878,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Didascalia grande in alto, MAIUSCOLO, carattere Anton stretto, su 2 righe. Prima immagine: la domanda principale. Sotto c'è la Home con i passi di oggi.</t>
+          <t>Didascalia grande in alto, MAIUSCOLO, carattere Anton stretto, su 2 righe. Prima immagine: la domanda principale. Sotto c'è la Home con i passi di oggi. Indica DOVE ANDARE A CAPO con « / » (es. «QUANTI PASSI / HAI FATTO OGGI?»): obbligatorio per JA/KO/ZH, utile per tutte.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -947,7 +954,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>MAIUSCOLO, 2 righe. Sotto: i minuti di camminata che mancano.</t>
+          <t>MAIUSCOLO, 2 righe. Sotto: i minuti di camminata che mancano. Indica DOVE ANDARE A CAPO con « / » (es. «QUANTI PASSI / HAI FATTO OGGI?»): obbligatorio per JA/KO/ZH, utile per tutte.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1023,7 +1030,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>MAIUSCOLO, 2 righe. Sotto: lo stesso giorno a 4 e a 16 km/h, i minuti cambiano.</t>
+          <t>MAIUSCOLO, 2 righe. Sotto: lo stesso giorno a 4 e a 16 km/h, i minuti cambiano. Indica DOVE ANDARE A CAPO con « / » (es. «QUANTI PASSI / HAI FATTO OGGI?»): obbligatorio per JA/KO/ZH, utile per tutte.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1099,7 +1106,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>MAIUSCOLO, 2 righe. Sotto: lo Storico con la serie (glossario).</t>
+          <t>MAIUSCOLO, 2 righe. Sotto: lo Storico con la serie (glossario). Indica DOVE ANDARE A CAPO con « / » (es. «QUANTI PASSI / HAI FATTO OGGI?»): obbligatorio per JA/KO/ZH, utile per tutte.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1175,7 +1182,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>MAIUSCOLO, 2 righe. Sotto: i widget.</t>
+          <t>MAIUSCOLO, 2 righe. Sotto: i widget. Indica DOVE ANDARE A CAPO con « / » (es. «QUANTI PASSI / HAI FATTO OGGI?»): obbligatorio per JA/KO/ZH, utile per tutte.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -1251,7 +1258,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>MAIUSCOLO, 2 righe. La promessa sulla privacy (stessa del testo promozionale).</t>
+          <t>MAIUSCOLO, 2 righe. La promessa sulla privacy (stessa del testo promozionale). Indica DOVE ANDARE A CAPO con « / » (es. «QUANTI PASSI / HAI FATTO OGGI?»): obbligatorio per JA/KO/ZH, utile per tutte.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1289,12 +1296,12 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Etichetta nera.</t>
+          <t>Etichetta nera. Non ripetere le tre etichette sotto (account, pubblicità, tracciamento).</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Niente account, niente pubblicità</t>
+          <t>Nessun dato lascia il telefono</t>
         </is>
       </c>
       <c r="F18" s="6" t="n"/>

</xml_diff>